<commit_message>
fix(timetable): correct native workbook evidence boundaries
</commit_message>
<xml_diff>
--- a/apps/api/test/fixtures/tkb/sanitized-dam-san-tkb-fixture.xlsx
+++ b/apps/api/test/fixtures/tkb/sanitized-dam-san-tkb-fixture.xlsx
@@ -106,181 +106,181 @@
     <t>2</t>
   </si>
   <si>
-    <t>TO-T2</t>
-  </si>
-  <si>
-    <t>TO-T1</t>
-  </si>
-  <si>
-    <t>NN-A2</t>
-  </si>
-  <si>
-    <t>TI-TN1</t>
-  </si>
-  <si>
-    <t>DI-Đ2</t>
-  </si>
-  <si>
-    <t>HO-H2</t>
-  </si>
-  <si>
-    <t>TI-TN2</t>
-  </si>
-  <si>
-    <t>LI-L2</t>
-  </si>
-  <si>
-    <t>SU-S2</t>
-  </si>
-  <si>
-    <t>VA-V3</t>
-  </si>
-  <si>
-    <t>DI-Đ1</t>
-  </si>
-  <si>
-    <t>CD-KP2</t>
-  </si>
-  <si>
-    <t>TO-T6</t>
-  </si>
-  <si>
-    <t>SI-SV2</t>
-  </si>
-  <si>
-    <t>CN-SV3</t>
-  </si>
-  <si>
-    <t>VA-V8</t>
-  </si>
-  <si>
-    <t>HO-H1</t>
-  </si>
-  <si>
-    <t>VA-V7</t>
+    <t>TO-GV02</t>
+  </si>
+  <si>
+    <t>TO-GV01</t>
+  </si>
+  <si>
+    <t>NN-GV33</t>
+  </si>
+  <si>
+    <t>TI-GV08</t>
+  </si>
+  <si>
+    <t>DI-GV31</t>
+  </si>
+  <si>
+    <t>HO-GV14</t>
+  </si>
+  <si>
+    <t>TI-GV09</t>
+  </si>
+  <si>
+    <t>LI-GV11</t>
+  </si>
+  <si>
+    <t>SU-GV27</t>
+  </si>
+  <si>
+    <t>VA-GV20</t>
+  </si>
+  <si>
+    <t>DI-GV30</t>
+  </si>
+  <si>
+    <t>CD-GV29</t>
+  </si>
+  <si>
+    <t>TO-GV06</t>
+  </si>
+  <si>
+    <t>SI-GV16</t>
+  </si>
+  <si>
+    <t>CN-GV17</t>
+  </si>
+  <si>
+    <t>VA-GV24</t>
+  </si>
+  <si>
+    <t>HO-GV13</t>
+  </si>
+  <si>
+    <t>VA-GV23</t>
   </si>
   <si>
     <t>3</t>
   </si>
   <si>
-    <t>LI-L3</t>
-  </si>
-  <si>
-    <t>VA-V5</t>
-  </si>
-  <si>
-    <t>NN-A5</t>
-  </si>
-  <si>
-    <t>SI-SV3</t>
-  </si>
-  <si>
-    <t>TO-T5</t>
-  </si>
-  <si>
-    <t>VA-V4</t>
-  </si>
-  <si>
-    <t>NN-A1</t>
-  </si>
-  <si>
-    <t>SU-S1</t>
-  </si>
-  <si>
-    <t>TO-T3</t>
+    <t>LI-GV12</t>
+  </si>
+  <si>
+    <t>VA-GV22</t>
+  </si>
+  <si>
+    <t>NN-GV34</t>
+  </si>
+  <si>
+    <t>SI-GV17</t>
+  </si>
+  <si>
+    <t>TO-GV05</t>
+  </si>
+  <si>
+    <t>VA-GV21</t>
+  </si>
+  <si>
+    <t>NN-GV32</t>
+  </si>
+  <si>
+    <t>SU-GV26</t>
+  </si>
+  <si>
+    <t>TO-GV03</t>
   </si>
   <si>
     <t>4</t>
   </si>
   <si>
-    <t>CN-L3</t>
-  </si>
-  <si>
-    <t>CN-L2</t>
-  </si>
-  <si>
-    <t>TO-T7</t>
-  </si>
-  <si>
-    <t>VA-V2</t>
-  </si>
-  <si>
-    <t>CN-SV1</t>
-  </si>
-  <si>
-    <t>TO-T4</t>
-  </si>
-  <si>
-    <t>LI-L1</t>
-  </si>
-  <si>
-    <t>CD-KP1</t>
-  </si>
-  <si>
-    <t>CN-L1</t>
-  </si>
-  <si>
-    <t>VA-V9</t>
-  </si>
-  <si>
-    <t>SI-SV1</t>
+    <t>CN-GV12</t>
+  </si>
+  <si>
+    <t>CN-GV11</t>
+  </si>
+  <si>
+    <t>TO-GV07</t>
+  </si>
+  <si>
+    <t>VA-GV19</t>
+  </si>
+  <si>
+    <t>CN-GV15</t>
+  </si>
+  <si>
+    <t>TO-GV04</t>
+  </si>
+  <si>
+    <t>LI-GV10</t>
+  </si>
+  <si>
+    <t>CD-GV28</t>
+  </si>
+  <si>
+    <t>CN-GV10</t>
+  </si>
+  <si>
+    <t>VA-GV25</t>
+  </si>
+  <si>
+    <t>SI-GV15</t>
   </si>
   <si>
     <t>GDĐP</t>
   </si>
   <si>
-    <t>SH-V4</t>
-  </si>
-  <si>
-    <t>SH-L3</t>
-  </si>
-  <si>
-    <t>SH-V8</t>
-  </si>
-  <si>
-    <t>SH-V5</t>
-  </si>
-  <si>
-    <t>SH-T5</t>
-  </si>
-  <si>
-    <t>SH-T1</t>
-  </si>
-  <si>
-    <t>SH-H1</t>
-  </si>
-  <si>
-    <t>SH-L2</t>
-  </si>
-  <si>
-    <t>SH-KP2</t>
-  </si>
-  <si>
-    <t>SH-T7</t>
-  </si>
-  <si>
-    <t>SH-Đ1</t>
-  </si>
-  <si>
-    <t>SH-SV3</t>
-  </si>
-  <si>
-    <t>SH-H2</t>
-  </si>
-  <si>
-    <t>SH-T2</t>
-  </si>
-  <si>
-    <t>SH-V3</t>
-  </si>
-  <si>
-    <t>SH-TN2</t>
-  </si>
-  <si>
-    <t>SH-SV2</t>
-  </si>
-  <si>
-    <t>SH-V7</t>
+    <t>SH-GV21</t>
+  </si>
+  <si>
+    <t>SH-GV12</t>
+  </si>
+  <si>
+    <t>SH-GV24</t>
+  </si>
+  <si>
+    <t>SH-GV22</t>
+  </si>
+  <si>
+    <t>SH-GV05</t>
+  </si>
+  <si>
+    <t>SH-GV01</t>
+  </si>
+  <si>
+    <t>SH-GV13</t>
+  </si>
+  <si>
+    <t>SH-GV11</t>
+  </si>
+  <si>
+    <t>SH-GV29</t>
+  </si>
+  <si>
+    <t>SH-GV07</t>
+  </si>
+  <si>
+    <t>SH-GV30</t>
+  </si>
+  <si>
+    <t>SH-GV17</t>
+  </si>
+  <si>
+    <t>SH-GV14</t>
+  </si>
+  <si>
+    <t>SH-GV02</t>
+  </si>
+  <si>
+    <t>SH-GV20</t>
+  </si>
+  <si>
+    <t>SH-GV09</t>
+  </si>
+  <si>
+    <t>SH-GV16</t>
+  </si>
+  <si>
+    <t>SH-GV23</t>
   </si>
   <si>
     <t>TN-HN</t>
@@ -466,19 +466,19 @@
     <t>THỜI KHOÁ BIỂU BUỔI CHIỀU NĂM HỌC 2026-2027 - ÁP DỤNG TỪ NGÀY 07/9/2026</t>
   </si>
   <si>
-    <t>TD-TD4</t>
-  </si>
-  <si>
-    <t>QP-TD5</t>
-  </si>
-  <si>
-    <t>TD-TD2</t>
-  </si>
-  <si>
-    <t>TD-TD5</t>
-  </si>
-  <si>
-    <t>QP-TD1</t>
+    <t>TD-GV37</t>
+  </si>
+  <si>
+    <t>QP-GV38</t>
+  </si>
+  <si>
+    <t>TD-GV36</t>
+  </si>
+  <si>
+    <t>TD-GV38</t>
+  </si>
+  <si>
+    <t>QP-GV35</t>
   </si>
   <si>
     <t>Giáo dục thế chất: TD, Giáo dục quốc phòng và an ninh: QP</t>

</xml_diff>